<commit_message>
added more data to my file
</commit_message>
<xml_diff>
--- a/Data/Data Second Assignment/DataPhase2Sharma.xlsx
+++ b/Data/Data Second Assignment/DataPhase2Sharma.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ssharma\CS424_Fall2016_Project\Data\Data Second Assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA41E4BC-D8A9-461C-A909-E175428DE8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29253A42-1565-4ECA-8E4C-0D7B1E0904B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="87">
   <si>
     <t>Date</t>
   </si>
@@ -238,6 +238,54 @@
   </si>
   <si>
     <t>Berwyn and Broadway (Red Line)</t>
+  </si>
+  <si>
+    <t>1 minute late; first observed bus</t>
+  </si>
+  <si>
+    <t>1 minute late; approximately 10-minute spacing</t>
+  </si>
+  <si>
+    <t>On time; next bus arrived sooner than predicted</t>
+  </si>
+  <si>
+    <t>Arrived earlier than predicted; possible bunching</t>
+  </si>
+  <si>
+    <t>Arrived shortly after previous bus; bunching observed</t>
+  </si>
+  <si>
+    <t>1 minute late; regular spacing</t>
+  </si>
+  <si>
+    <t>1 minute late; slightly longer following interval</t>
+  </si>
+  <si>
+    <t>3 minutes late; service remains relatively regular</t>
+  </si>
+  <si>
+    <t>2 minutes late; approximately 19-minute interval since previous bus</t>
+  </si>
+  <si>
+    <t>1 minute late; approximately regular spacing</t>
+  </si>
+  <si>
+    <t>On time; regular spacing</t>
+  </si>
+  <si>
+    <t>1 minute late; no substantial bunching observed</t>
+  </si>
+  <si>
+    <t>1 minute late; approximately 20-minute spacing</t>
+  </si>
+  <si>
+    <t>Bus bunching observed; followed by a long service gap</t>
+  </si>
+  <si>
+    <t>Approximately 27-minute service gap; bus arrived later than predicted</t>
+  </si>
+  <si>
+    <t>Bus closely followed previous bus; another bunching episode</t>
   </si>
 </sst>
 </file>
@@ -2277,7 +2325,7 @@
         <v>46308</v>
       </c>
       <c r="C42" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D42">
         <v>36</v>
@@ -2290,6 +2338,24 @@
       </c>
       <c r="G42" t="s">
         <v>15</v>
+      </c>
+      <c r="H42" s="3">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="I42" s="3">
+        <v>0.33402777777777776</v>
+      </c>
+      <c r="J42" t="s">
+        <v>16</v>
+      </c>
+      <c r="K42">
+        <v>10</v>
+      </c>
+      <c r="L42">
+        <v>10</v>
+      </c>
+      <c r="M42" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
@@ -2314,6 +2380,24 @@
       <c r="G43" t="s">
         <v>15</v>
       </c>
+      <c r="H43" s="3">
+        <v>0.34027777777777779</v>
+      </c>
+      <c r="I43" s="3">
+        <v>0.34097222222222223</v>
+      </c>
+      <c r="J43">
+        <v>10</v>
+      </c>
+      <c r="K43">
+        <v>10</v>
+      </c>
+      <c r="L43">
+        <v>9</v>
+      </c>
+      <c r="M43" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44">
@@ -2337,6 +2421,24 @@
       <c r="G44" t="s">
         <v>15</v>
       </c>
+      <c r="H44" s="3">
+        <v>0.34722222222222221</v>
+      </c>
+      <c r="I44" s="3">
+        <v>0.34722222222222221</v>
+      </c>
+      <c r="J44">
+        <v>9</v>
+      </c>
+      <c r="K44">
+        <v>10</v>
+      </c>
+      <c r="L44">
+        <v>3</v>
+      </c>
+      <c r="M44" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45">
@@ -2360,6 +2462,24 @@
       <c r="G45" t="s">
         <v>15</v>
       </c>
+      <c r="H45" s="3">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="I45" s="3">
+        <v>0.34930555555555554</v>
+      </c>
+      <c r="J45">
+        <v>3</v>
+      </c>
+      <c r="K45">
+        <v>10</v>
+      </c>
+      <c r="L45">
+        <v>4</v>
+      </c>
+      <c r="M45" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46">
@@ -2383,6 +2503,24 @@
       <c r="G46" t="s">
         <v>15</v>
       </c>
+      <c r="H46" s="3">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="I46" s="3">
+        <v>0.35208333333333336</v>
+      </c>
+      <c r="J46">
+        <v>4</v>
+      </c>
+      <c r="K46" t="s">
+        <v>16</v>
+      </c>
+      <c r="L46" t="s">
+        <v>16</v>
+      </c>
+      <c r="M46" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47">
@@ -2406,6 +2544,24 @@
       <c r="G47" t="s">
         <v>15</v>
       </c>
+      <c r="H47" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I47" s="3">
+        <v>0.50069444444444444</v>
+      </c>
+      <c r="J47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K47">
+        <v>20</v>
+      </c>
+      <c r="L47">
+        <v>20</v>
+      </c>
+      <c r="M47" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48">
@@ -2429,8 +2585,26 @@
       <c r="G48" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H48" s="3">
+        <v>0.51388888888888884</v>
+      </c>
+      <c r="I48" s="3">
+        <v>0.51458333333333328</v>
+      </c>
+      <c r="J48">
+        <v>20</v>
+      </c>
+      <c r="K48">
+        <v>20</v>
+      </c>
+      <c r="L48">
+        <v>20</v>
+      </c>
+      <c r="M48" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2452,8 +2626,26 @@
       <c r="G49" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H49" s="3">
+        <v>0.52777777777777779</v>
+      </c>
+      <c r="I49" s="3">
+        <v>0.52847222222222223</v>
+      </c>
+      <c r="J49">
+        <v>20</v>
+      </c>
+      <c r="K49">
+        <v>20</v>
+      </c>
+      <c r="L49">
+        <v>22</v>
+      </c>
+      <c r="M49" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2475,8 +2667,26 @@
       <c r="G50" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H50" s="3">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="I50" s="3">
+        <v>0.54374999999999996</v>
+      </c>
+      <c r="J50">
+        <v>22</v>
+      </c>
+      <c r="K50">
+        <v>20</v>
+      </c>
+      <c r="L50">
+        <v>19</v>
+      </c>
+      <c r="M50" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2498,8 +2708,26 @@
       <c r="G51" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H51" s="3">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="I51" s="3">
+        <v>0.55694444444444446</v>
+      </c>
+      <c r="J51">
+        <v>19</v>
+      </c>
+      <c r="K51" t="s">
+        <v>16</v>
+      </c>
+      <c r="L51" t="s">
+        <v>16</v>
+      </c>
+      <c r="M51" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2521,8 +2749,26 @@
       <c r="G52" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H52" s="3">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="I52" s="3">
+        <v>0.70902777777777781</v>
+      </c>
+      <c r="J52" t="s">
+        <v>16</v>
+      </c>
+      <c r="K52">
+        <v>20</v>
+      </c>
+      <c r="L52">
+        <v>20</v>
+      </c>
+      <c r="M52" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2544,8 +2790,26 @@
       <c r="G53" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H53" s="3">
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="I53" s="3">
+        <v>0.72291666666666665</v>
+      </c>
+      <c r="J53">
+        <v>20</v>
+      </c>
+      <c r="K53">
+        <v>20</v>
+      </c>
+      <c r="L53">
+        <v>19</v>
+      </c>
+      <c r="M53" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2567,8 +2831,26 @@
       <c r="G54" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H54" s="3">
+        <v>0.73611111111111116</v>
+      </c>
+      <c r="I54" s="3">
+        <v>0.73611111111111116</v>
+      </c>
+      <c r="J54">
+        <v>19</v>
+      </c>
+      <c r="K54">
+        <v>20</v>
+      </c>
+      <c r="L54">
+        <v>21</v>
+      </c>
+      <c r="M54" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2590,8 +2872,26 @@
       <c r="G55" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H55" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="I55" s="3">
+        <v>0.75069444444444444</v>
+      </c>
+      <c r="J55">
+        <v>21</v>
+      </c>
+      <c r="K55">
+        <v>20</v>
+      </c>
+      <c r="L55">
+        <v>20</v>
+      </c>
+      <c r="M55" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2613,8 +2913,26 @@
       <c r="G56" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H56" s="3">
+        <v>0.76388888888888884</v>
+      </c>
+      <c r="I56" s="3">
+        <v>0.76458333333333328</v>
+      </c>
+      <c r="J56">
+        <v>20</v>
+      </c>
+      <c r="K56" t="s">
+        <v>16</v>
+      </c>
+      <c r="L56" t="s">
+        <v>16</v>
+      </c>
+      <c r="M56" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2636,8 +2954,26 @@
       <c r="G57" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H57" s="3">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="I57" s="3">
+        <v>0.83402777777777781</v>
+      </c>
+      <c r="J57" t="s">
+        <v>16</v>
+      </c>
+      <c r="K57">
+        <v>12</v>
+      </c>
+      <c r="L57">
+        <v>3</v>
+      </c>
+      <c r="M57" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2659,8 +2995,26 @@
       <c r="G58" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H58" s="3">
+        <v>0.84166666666666667</v>
+      </c>
+      <c r="I58" s="3">
+        <v>0.83611111111111114</v>
+      </c>
+      <c r="J58">
+        <v>3</v>
+      </c>
+      <c r="K58">
+        <v>10</v>
+      </c>
+      <c r="L58">
+        <v>2</v>
+      </c>
+      <c r="M58" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2682,8 +3036,26 @@
       <c r="G59" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H59" s="3">
+        <v>0.84861111111111109</v>
+      </c>
+      <c r="I59" s="3">
+        <v>0.83750000000000002</v>
+      </c>
+      <c r="J59">
+        <v>2</v>
+      </c>
+      <c r="K59">
+        <v>12</v>
+      </c>
+      <c r="L59">
+        <v>27</v>
+      </c>
+      <c r="M59" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2705,8 +3077,26 @@
       <c r="G60" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H60" s="3">
+        <v>0.84583333333333333</v>
+      </c>
+      <c r="I60" s="3">
+        <v>0.85624999999999996</v>
+      </c>
+      <c r="J60">
+        <v>27</v>
+      </c>
+      <c r="K60">
+        <v>12</v>
+      </c>
+      <c r="L60">
+        <v>3</v>
+      </c>
+      <c r="M60" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2727,6 +3117,24 @@
       </c>
       <c r="G61" t="s">
         <v>14</v>
+      </c>
+      <c r="H61" s="3">
+        <v>0.86458333333333337</v>
+      </c>
+      <c r="I61" s="3">
+        <v>0.85833333333333328</v>
+      </c>
+      <c r="J61">
+        <v>3</v>
+      </c>
+      <c r="K61" t="s">
+        <v>16</v>
+      </c>
+      <c r="L61" t="s">
+        <v>16</v>
+      </c>
+      <c r="M61" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>